<commit_message>
setup limits on biostuff
</commit_message>
<xml_diff>
--- a/data/carriers_data/methane_bio/methane_bio_availability.xlsx
+++ b/data/carriers_data/methane_bio/methane_bio_availability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\carriers_data\methane_bio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A031274-0766-41A6-8EA6-53966F2615DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC501E9D-21C0-464F-8F4F-C08E0BE213F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16620" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="note" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>BE</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>availability in bcm/y</t>
-  </si>
-  <si>
-    <t>Weights on availability (source: https://en.wikipedia.org/wiki/List_of_countries_by_natural_gas_consumption)</t>
   </si>
   <si>
     <t>EU</t>
@@ -381,34 +378,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1">
-        <v>0.04</v>
-      </c>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="1">
-        <v>0.05</v>
-      </c>
+      <c r="B6" s="1"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="1">
-        <v>0.08</v>
-      </c>
+      <c r="B7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -422,7 +399,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B1">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C1">
         <v>2030</v>
@@ -439,20 +416,18 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <f>note!$B5*availability!B$5</f>
-        <v>0.88</v>
+        <f>C2</f>
+        <v>0.5</v>
       </c>
       <c r="C2">
-        <f>note!$B$5*availability!C$5</f>
-        <v>1.4000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="D2">
-        <f>note!$B$5*availability!D$5</f>
-        <v>4.8</v>
+        <f t="shared" ref="D2:D4" si="0">AVERAGE(C2,E2)</f>
+        <v>1</v>
       </c>
       <c r="E2">
-        <f>note!$B$5*availability!E$5</f>
-        <v>7.6000000000000005</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -460,20 +435,18 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <f>note!$B6*availability!B$5</f>
-        <v>1.1000000000000001</v>
+        <f t="shared" ref="B3:B4" si="1">C3</f>
+        <v>7.5</v>
       </c>
       <c r="C3">
-        <f>note!$B$5*availability!C$5</f>
-        <v>1.4000000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="D3">
-        <f>note!$B$5*availability!D$5</f>
-        <v>4.8</v>
+        <f t="shared" si="0"/>
+        <v>14.75</v>
       </c>
       <c r="E3">
-        <f>note!$B$5*availability!E$5</f>
-        <v>7.6000000000000005</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -481,37 +454,36 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <f>note!$B7*availability!B$5</f>
-        <v>1.76</v>
+        <f t="shared" si="1"/>
+        <v>1.5</v>
       </c>
       <c r="C4">
-        <f>note!$B$5*availability!C$5</f>
-        <v>1.4000000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="D4">
-        <f>note!$B$5*availability!D$5</f>
-        <v>4.8</v>
+        <f t="shared" si="0"/>
+        <v>2.5</v>
       </c>
       <c r="E4">
-        <f>note!$B$5*availability!E$5</f>
-        <v>7.6000000000000005</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="C5">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D5">
-        <v>120</v>
+        <f>AVERAGE(C5,E5)</f>
+        <v>96</v>
       </c>
       <c r="E5">
-        <v>190</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>